<commit_message>
Audit lower pins and electrical gates; repair BOM overlay
</commit_message>
<xml_diff>
--- a/outputs/20261002_reve_followthrough/2026_BIZ-Lab_재료비관리_RevE_연속검수.xlsx
+++ b/outputs/20261002_reve_followthrough/2026_BIZ-Lab_재료비관리_RevE_연속검수.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R2810baf9fd3446b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Raddd6bd44a3d4abf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -276,52 +276,6 @@
 </x:styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>1924050</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="1" name="Text Box 2"/>
-        <xdr:cNvSpPr>
-          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="0" y="0"/>
-          <a:ext cx="9525000" cy="9525000"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:srgbClr val="FFFFFF"/>
-        </a:solidFill>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-          <a:miter/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
@@ -1214,7 +1168,7 @@
         <x:v>20990</x:v>
       </x:c>
       <x:c r="I26" s="5" t="str">
-        <x:v>E08. VAT 포함 표시가를 공급가로 환산. 재고·배송비·최종 결제금액 확인.</x:v>
+        <x:v>E08. 출하표시 10/06과 배송까지 3개월 이상 가능 경고가 상충. 11월 말 일정용 확정 납기 아님. 실제 납기·보호곡선 확인 전 발주 보류.</x:v>
       </x:c>
       <x:c r="M26" s="1"/>
     </x:row>
@@ -1617,7 +1571,7 @@
         <x:v>6600</x:v>
       </x:c>
       <x:c r="I41" s="5" t="str">
-        <x:v>E10. VAT 포함 표시가를 공급가로 환산. 재고·배송비·최종 결제금액 확인.</x:v>
+        <x:v>E10. 현재 STOP 스위치의 직접개리·DC-13 정격 미확인. 24 V 접촉기 코일 차단용 승인 전까지 주문·통전 보류.</x:v>
       </x:c>
       <x:c r="M41" s="1"/>
     </x:row>
@@ -2049,7 +2003,7 @@
         <x:v>12000</x:v>
       </x:c>
       <x:c r="I57" s="5" t="str">
-        <x:v>M02. VAT 포함 표시가를 공급가로 환산. 재고·배송비·최종 결제금액 확인.</x:v>
+        <x:v>M02. 사진에는 핀·R클립이 보이나 단일옵션 동봉 수량 미명시. 3세트 각 1조 확보, 눈홀 판매도면 Ø6.4/STEP Ø6.0 불일치·측면 유격 확인 전 조립 보류.</x:v>
       </x:c>
       <x:c r="M57" s="1"/>
     </x:row>
@@ -8881,75 +8835,74 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="Rff10ca6424884d0d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="R74779e7b25104aa0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="R724c182826634297"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="R2fc471276225456e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="R91efa326ede14dec"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="R602b2d3f791a482c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="R0875cb7763e44099"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="R9c1fcd3580d942a0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="Rf049a9cc31de46ba"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="R256318cb7a2d4cbf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="Ref432266cb134ece"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="Rdc61743f4e034719"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="R31b95ebf81e54bfb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="R5473c2e3f0c64e2e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="R6dcc813257b247f3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="R632dd1f780fa4b7f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="R6098bb842146423e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="Re95fa50003f14838"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="R4d9d975bfc994950"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="R336ce1c7016b49a6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="Rb5ee9e4c280844ae"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="R02919b4bcc8d45ec"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="Ra80439215f214055"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="Re72979fcd7224f2b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="Rc7782fca2cb745e0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="R6e72aa57b23b4155"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="R896e33eff3f24704"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="R07238cacd91545dd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="R15a12d93fb444b47"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="Raf51870ae649493c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R2b8425e260204fb9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="R915f33b35f8e4149"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="R246eb792b2494deb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="Rfcf419059ee24cd3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="R4b83dbbb13d84750"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="Red0c2eee63e54812"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="Rca8c64d238ad4858"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="R0fb642460934412e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="Rd80c191b75ef4a8f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="R902b09a875794c8e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="R7f06badd017a4146"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="R4a5b05aba6994472"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="R44f5510ce06a4a0f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="Rde77d3e9f28244fc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="Rf04d5b05579c49d8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="R9b43cc58f4ee4dc7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="Ra6fa5c327bb848ea"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="Rb02104e508ed4ed5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="R70f709bfeb5f4fb3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="R37eb0eb3985e47ce"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="Rfaf971f33a274493"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="R9bce339217764b96"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="R7c0f1f9c6a0e4ff3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="Rdbdf63cc0a604141"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="R38570cf88e0c46ec"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="Rabb82bff747c4021"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="Rb5493bda13d94854"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="R2726fb8007544b03"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="R124ac6bd72a644f6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="R50e7bdf110b745dd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="Rf922f11968794b2e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="Re7b14bfafd804b36"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="R62b8f5c8e4984153"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="R73c72b36df514299"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="R028869e28a9c459e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="R33ca0ee6e6a04407"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="R819ba44cf3374269"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="R5d04fb0fca1a4446"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="R7260aae113274dee"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="R7517b8e0cc414c0b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="R63a8b9f41b8f44a9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="R782be107a7fc4ac2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="R56690ae308c2432a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="Rbcc0a9d70e0a4bb7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="R994b006878d04a57"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="R2b7e3f27c1e54141"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="R8be8bff2d58f49c5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="Rb2a1f8eb8dcc414f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="R3f15c539c05244aa"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="R9b08128879a24fd0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="Rd35920f922cf44ac"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="R3fd2b340835f435b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="R32ff215b265441c0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="Recb418f8ed284b79"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="Rc44834245d8d4ece"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="Rf0cbff99231e4fd5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="R2b01c89ad6da4183"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="Racb260ece7e24dec"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="R086fdad9f4e84204"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="R2a153748da5748f0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="R5d1aa085c311463f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="R979eb96637124d77"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="R610fc529d0c74cd0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="R93c08016c7464d4c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="Ra1d6b4e359e04cc6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="Rb6044785173f4dba"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="R887c5a1dcb6142e5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R9661d78f55494f48"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="R1f94eafcc4984c45"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="R82e07d055452409a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="R2cafb43e09214d44"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="Rbc1169430c53400c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="R199d50e1009a493f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="R39a29b2c61024f37"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="R95ae772a8e15492c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="R2c8d7b4575b84152"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="Rcd825a59d0984f93"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="Re81c153ef8604c95"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="Rd2212ca7592b416b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="R1e5301f529564792"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="R54f926507b6b4b57"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="Rdeee6057e4f44226"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="R58248cb8e59b46d7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="R624879a202604d16"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="R185ea91ea6f74ea7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="Rbbbb4f988e584c88"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="R485294588a1144d3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="Rd5df235c8d5c438e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="R66f54892a70e4673"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="Rcde1cdbd53f04fe2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="R168661d3a8a34e91"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="R5c08fb6f4daa4622"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="R58041cce139c4ae4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="R3e39380af24f467b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="R26ade0598c864a70"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="Rc4f71f3ea67040a9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="R2b85dcd04c8846dc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="R1268bf3a806d44f8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="R0f86f9b878ac40ee"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="Rb10144d487244f69"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="Rf05e70d7ac9f4ebf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="R53fab6727d874a72"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="R61df7b81f32945bb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="R63a07f4aa2d54315"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28d2e6e42b264119"/>
 </x:worksheet>
 </file>
</xml_diff>